<commit_message>
Listino: rimuovi kit, filo infinito e ricarica doppia Filo Coraggioso
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01J4R9p7aLyjCzNEo4SKhjXF
</commit_message>
<xml_diff>
--- a/listini/Listino_Vivibiotic_2026-10.xlsx
+++ b/listini/Listino_Vivibiotic_2026-10.xlsx
@@ -470,7 +470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E32"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -677,11 +677,7 @@
           <t>Ricarica per Filo Coraggioso</t>
         </is>
       </c>
-      <c r="B14" s="9" t="inlineStr">
-        <is>
-          <t>Una ricarica</t>
-        </is>
-      </c>
+      <c r="B14" s="9" t="inlineStr"/>
       <c r="C14" s="10" t="n">
         <v>6.8</v>
       </c>
@@ -694,16 +690,12 @@
     <row r="15">
       <c r="A15" s="9" t="inlineStr">
         <is>
-          <t>Ricarica per Filo Coraggioso</t>
-        </is>
-      </c>
-      <c r="B15" s="9" t="inlineStr">
-        <is>
-          <t>Due ricariche</t>
-        </is>
-      </c>
+          <t>Ricarica per filo infinito 250 m</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="inlineStr"/>
       <c r="C15" s="10" t="n">
-        <v>12.5</v>
+        <v>60</v>
       </c>
       <c r="D15" s="11">
         <f>ROUND(C15*(1-$E$2),2)</f>
@@ -712,30 +704,25 @@
       <c r="E15" s="9" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="9" t="inlineStr">
-        <is>
-          <t>Filo interdentale infinito</t>
-        </is>
-      </c>
-      <c r="B16" s="9" t="inlineStr"/>
-      <c r="C16" s="10" t="n">
-        <v>85</v>
-      </c>
-      <c r="D16" s="11">
-        <f>ROUND(C16*(1-$E$2),2)</f>
-        <v/>
-      </c>
-      <c r="E16" s="9" t="n"/>
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>OLI E CREME</t>
+        </is>
+      </c>
+      <c r="B16" s="8" t="n"/>
+      <c r="C16" s="8" t="n"/>
+      <c r="D16" s="8" t="n"/>
+      <c r="E16" s="8" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="9" t="inlineStr">
         <is>
-          <t>Ricarica per filo infinito 250 m</t>
+          <t>Olio Favoloso 100 ml</t>
         </is>
       </c>
       <c r="B17" s="9" t="inlineStr"/>
       <c r="C17" s="10" t="n">
-        <v>60</v>
+        <v>45</v>
       </c>
       <c r="D17" s="11">
         <f>ROUND(C17*(1-$E$2),2)</f>
@@ -744,25 +731,30 @@
       <c r="E17" s="9" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="7" t="inlineStr">
-        <is>
-          <t>OLI E CREME</t>
-        </is>
-      </c>
-      <c r="B18" s="8" t="n"/>
-      <c r="C18" s="8" t="n"/>
-      <c r="D18" s="8" t="n"/>
-      <c r="E18" s="8" t="n"/>
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t>L'Olio Adorabile 125 ml</t>
+        </is>
+      </c>
+      <c r="B18" s="9" t="inlineStr"/>
+      <c r="C18" s="10" t="n">
+        <v>75</v>
+      </c>
+      <c r="D18" s="11">
+        <f>ROUND(C18*(1-$E$2),2)</f>
+        <v/>
+      </c>
+      <c r="E18" s="9" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="9" t="inlineStr">
         <is>
-          <t>Olio Favoloso 100 ml</t>
+          <t>Tattoo Cream 50 ml</t>
         </is>
       </c>
       <c r="B19" s="9" t="inlineStr"/>
       <c r="C19" s="10" t="n">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="D19" s="11">
         <f>ROUND(C19*(1-$E$2),2)</f>
@@ -771,30 +763,25 @@
       <c r="E19" s="9" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="9" t="inlineStr">
-        <is>
-          <t>L'Olio Adorabile 125 ml</t>
-        </is>
-      </c>
-      <c r="B20" s="9" t="inlineStr"/>
-      <c r="C20" s="10" t="n">
-        <v>75</v>
-      </c>
-      <c r="D20" s="11">
-        <f>ROUND(C20*(1-$E$2),2)</f>
-        <v/>
-      </c>
-      <c r="E20" s="9" t="n"/>
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>LIBRI E ACCESSORI</t>
+        </is>
+      </c>
+      <c r="B20" s="8" t="n"/>
+      <c r="C20" s="8" t="n"/>
+      <c r="D20" s="8" t="n"/>
+      <c r="E20" s="8" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="9" t="inlineStr">
         <is>
-          <t>Tattoo Cream 50 ml</t>
+          <t>Missione Denti: libro per bambini e genitori</t>
         </is>
       </c>
       <c r="B21" s="9" t="inlineStr"/>
       <c r="C21" s="10" t="n">
-        <v>39</v>
+        <v>15</v>
       </c>
       <c r="D21" s="11">
         <f>ROUND(C21*(1-$E$2),2)</f>
@@ -803,25 +790,30 @@
       <c r="E21" s="9" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="7" t="inlineStr">
-        <is>
-          <t>KIT</t>
-        </is>
-      </c>
-      <c r="B22" s="8" t="n"/>
-      <c r="C22" s="8" t="n"/>
-      <c r="D22" s="8" t="n"/>
-      <c r="E22" s="8" t="n"/>
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>Ebook - La Bocca Ormonale</t>
+        </is>
+      </c>
+      <c r="B22" s="9" t="inlineStr"/>
+      <c r="C22" s="10" t="n">
+        <v>9.9</v>
+      </c>
+      <c r="D22" s="11">
+        <f>ROUND(C22*(1-$E$2),2)</f>
+        <v/>
+      </c>
+      <c r="E22" s="9" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="9" t="inlineStr">
         <is>
-          <t>Kit Starter: tutto il necessario per un sorriso sano</t>
+          <t>Borsa Kit Vivibiotic</t>
         </is>
       </c>
       <c r="B23" s="9" t="inlineStr"/>
       <c r="C23" s="10" t="n">
-        <v>60</v>
+        <v>5</v>
       </c>
       <c r="D23" s="11">
         <f>ROUND(C23*(1-$E$2),2)</f>
@@ -829,172 +821,25 @@
       </c>
       <c r="E23" s="9" t="n"/>
     </row>
-    <row r="24">
-      <c r="A24" s="9" t="inlineStr">
-        <is>
-          <t>Kit Keto: Collutorio + Dentifricio + Spazzolino</t>
-        </is>
-      </c>
-      <c r="B24" s="9" t="inlineStr"/>
-      <c r="C24" s="10" t="n">
-        <v>46.5</v>
-      </c>
-      <c r="D24" s="11">
-        <f>ROUND(C24*(1-$E$2),2)</f>
-        <v/>
-      </c>
-      <c r="E24" s="9" t="n"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="9" t="inlineStr">
-        <is>
-          <t>Kit Giorno e Notte</t>
-        </is>
-      </c>
-      <c r="B25" s="9" t="inlineStr"/>
-      <c r="C25" s="10" t="n">
-        <v>37.91</v>
-      </c>
-      <c r="D25" s="11">
-        <f>ROUND(C25*(1-$E$2),2)</f>
-        <v/>
-      </c>
-      <c r="E25" s="9" t="n"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="9" t="inlineStr">
-        <is>
-          <t>Kit Esoso</t>
-        </is>
-      </c>
-      <c r="B26" s="9" t="inlineStr"/>
-      <c r="C26" s="10" t="n">
-        <v>39.6</v>
-      </c>
-      <c r="D26" s="11">
-        <f>ROUND(C26*(1-$E$2),2)</f>
-        <v/>
-      </c>
-      <c r="E26" s="9" t="n"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="9" t="inlineStr">
-        <is>
-          <t>Kit La Bocca Ormonale</t>
-        </is>
-      </c>
-      <c r="B27" s="9" t="inlineStr"/>
-      <c r="C27" s="10" t="n">
-        <v>44.9</v>
-      </c>
-      <c r="D27" s="11">
-        <f>ROUND(C27*(1-$E$2),2)</f>
-        <v/>
-      </c>
-      <c r="E27" s="9" t="n"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="9" t="inlineStr">
-        <is>
-          <t>Filo infinito + Ricarica 250 m</t>
-        </is>
-      </c>
-      <c r="B28" s="9" t="inlineStr"/>
-      <c r="C28" s="10" t="n">
-        <v>130</v>
-      </c>
-      <c r="D28" s="11">
-        <f>ROUND(C28*(1-$E$2),2)</f>
-        <v/>
-      </c>
-      <c r="E28" s="9" t="n"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="7" t="inlineStr">
-        <is>
-          <t>LIBRI E ACCESSORI</t>
-        </is>
-      </c>
-      <c r="B29" s="8" t="n"/>
-      <c r="C29" s="8" t="n"/>
-      <c r="D29" s="8" t="n"/>
-      <c r="E29" s="8" t="n"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="9" t="inlineStr">
-        <is>
-          <t>Missione Denti: libro per bambini e genitori</t>
-        </is>
-      </c>
-      <c r="B30" s="9" t="inlineStr"/>
-      <c r="C30" s="10" t="n">
-        <v>15</v>
-      </c>
-      <c r="D30" s="11">
-        <f>ROUND(C30*(1-$E$2),2)</f>
-        <v/>
-      </c>
-      <c r="E30" s="9" t="n"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="9" t="inlineStr">
-        <is>
-          <t>Ebook - La Bocca Ormonale</t>
-        </is>
-      </c>
-      <c r="B31" s="9" t="inlineStr"/>
-      <c r="C31" s="10" t="n">
-        <v>9.9</v>
-      </c>
-      <c r="D31" s="11">
-        <f>ROUND(C31*(1-$E$2),2)</f>
-        <v/>
-      </c>
-      <c r="E31" s="9" t="n"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="9" t="inlineStr">
-        <is>
-          <t>Borsa Kit Vivibiotic</t>
-        </is>
-      </c>
-      <c r="B32" s="9" t="inlineStr"/>
-      <c r="C32" s="10" t="n">
-        <v>5</v>
-      </c>
-      <c r="D32" s="11">
-        <f>ROUND(C32*(1-$E$2),2)</f>
-        <v/>
-      </c>
-      <c r="E32" s="9" t="n"/>
-    </row>
   </sheetData>
-  <mergeCells count="25">
-    <mergeCell ref="D20:E20"/>
+  <mergeCells count="17">
+    <mergeCell ref="D8:E8"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="D7:E7"/>
     <mergeCell ref="D10:E10"/>
+    <mergeCell ref="D15:E15"/>
     <mergeCell ref="D19:E19"/>
-    <mergeCell ref="D31:E31"/>
-    <mergeCell ref="D21:E21"/>
-    <mergeCell ref="D6:E6"/>
     <mergeCell ref="D11:E11"/>
     <mergeCell ref="D13:E13"/>
-    <mergeCell ref="D27:E27"/>
-    <mergeCell ref="D32:E32"/>
     <mergeCell ref="D17:E17"/>
-    <mergeCell ref="D16:E16"/>
-    <mergeCell ref="D7:E7"/>
-    <mergeCell ref="D28:E28"/>
+    <mergeCell ref="D23:E23"/>
+    <mergeCell ref="D14:E14"/>
     <mergeCell ref="D4:E4"/>
+    <mergeCell ref="D22:E22"/>
+    <mergeCell ref="D18:E18"/>
     <mergeCell ref="D9:E9"/>
     <mergeCell ref="D12:E12"/>
-    <mergeCell ref="D8:E8"/>
-    <mergeCell ref="D25:E25"/>
-    <mergeCell ref="D24:E24"/>
-    <mergeCell ref="D30:E30"/>
-    <mergeCell ref="D15:E15"/>
-    <mergeCell ref="D23:E23"/>
-    <mergeCell ref="D14:E14"/>
-    <mergeCell ref="D26:E26"/>
+    <mergeCell ref="D21:E21"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
Listino: rimuovi libri/accessori e ricarica filo infinito
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01J4R9p7aLyjCzNEo4SKhjXF
</commit_message>
<xml_diff>
--- a/listini/Listino_Vivibiotic_2026-10.xlsx
+++ b/listini/Listino_Vivibiotic_2026-10.xlsx
@@ -470,7 +470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -688,41 +688,41 @@
       <c r="E14" s="9" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="9" t="inlineStr">
-        <is>
-          <t>Ricarica per filo infinito 250 m</t>
-        </is>
-      </c>
-      <c r="B15" s="9" t="inlineStr"/>
-      <c r="C15" s="10" t="n">
-        <v>60</v>
-      </c>
-      <c r="D15" s="11">
-        <f>ROUND(C15*(1-$E$2),2)</f>
-        <v/>
-      </c>
-      <c r="E15" s="9" t="n"/>
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>OLI E CREME</t>
+        </is>
+      </c>
+      <c r="B15" s="8" t="n"/>
+      <c r="C15" s="8" t="n"/>
+      <c r="D15" s="8" t="n"/>
+      <c r="E15" s="8" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="7" t="inlineStr">
-        <is>
-          <t>OLI E CREME</t>
-        </is>
-      </c>
-      <c r="B16" s="8" t="n"/>
-      <c r="C16" s="8" t="n"/>
-      <c r="D16" s="8" t="n"/>
-      <c r="E16" s="8" t="n"/>
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>Olio Favoloso 100 ml</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="inlineStr"/>
+      <c r="C16" s="10" t="n">
+        <v>45</v>
+      </c>
+      <c r="D16" s="11">
+        <f>ROUND(C16*(1-$E$2),2)</f>
+        <v/>
+      </c>
+      <c r="E16" s="9" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="9" t="inlineStr">
         <is>
-          <t>Olio Favoloso 100 ml</t>
+          <t>L'Olio Adorabile 125 ml</t>
         </is>
       </c>
       <c r="B17" s="9" t="inlineStr"/>
       <c r="C17" s="10" t="n">
-        <v>45</v>
+        <v>75</v>
       </c>
       <c r="D17" s="11">
         <f>ROUND(C17*(1-$E$2),2)</f>
@@ -733,12 +733,12 @@
     <row r="18">
       <c r="A18" s="9" t="inlineStr">
         <is>
-          <t>L'Olio Adorabile 125 ml</t>
+          <t>Tattoo Cream 50 ml</t>
         </is>
       </c>
       <c r="B18" s="9" t="inlineStr"/>
       <c r="C18" s="10" t="n">
-        <v>75</v>
+        <v>39</v>
       </c>
       <c r="D18" s="11">
         <f>ROUND(C18*(1-$E$2),2)</f>
@@ -746,100 +746,21 @@
       </c>
       <c r="E18" s="9" t="n"/>
     </row>
-    <row r="19">
-      <c r="A19" s="9" t="inlineStr">
-        <is>
-          <t>Tattoo Cream 50 ml</t>
-        </is>
-      </c>
-      <c r="B19" s="9" t="inlineStr"/>
-      <c r="C19" s="10" t="n">
-        <v>39</v>
-      </c>
-      <c r="D19" s="11">
-        <f>ROUND(C19*(1-$E$2),2)</f>
-        <v/>
-      </c>
-      <c r="E19" s="9" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="7" t="inlineStr">
-        <is>
-          <t>LIBRI E ACCESSORI</t>
-        </is>
-      </c>
-      <c r="B20" s="8" t="n"/>
-      <c r="C20" s="8" t="n"/>
-      <c r="D20" s="8" t="n"/>
-      <c r="E20" s="8" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="9" t="inlineStr">
-        <is>
-          <t>Missione Denti: libro per bambini e genitori</t>
-        </is>
-      </c>
-      <c r="B21" s="9" t="inlineStr"/>
-      <c r="C21" s="10" t="n">
-        <v>15</v>
-      </c>
-      <c r="D21" s="11">
-        <f>ROUND(C21*(1-$E$2),2)</f>
-        <v/>
-      </c>
-      <c r="E21" s="9" t="n"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="9" t="inlineStr">
-        <is>
-          <t>Ebook - La Bocca Ormonale</t>
-        </is>
-      </c>
-      <c r="B22" s="9" t="inlineStr"/>
-      <c r="C22" s="10" t="n">
-        <v>9.9</v>
-      </c>
-      <c r="D22" s="11">
-        <f>ROUND(C22*(1-$E$2),2)</f>
-        <v/>
-      </c>
-      <c r="E22" s="9" t="n"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="9" t="inlineStr">
-        <is>
-          <t>Borsa Kit Vivibiotic</t>
-        </is>
-      </c>
-      <c r="B23" s="9" t="inlineStr"/>
-      <c r="C23" s="10" t="n">
-        <v>5</v>
-      </c>
-      <c r="D23" s="11">
-        <f>ROUND(C23*(1-$E$2),2)</f>
-        <v/>
-      </c>
-      <c r="E23" s="9" t="n"/>
-    </row>
   </sheetData>
-  <mergeCells count="17">
+  <mergeCells count="13">
     <mergeCell ref="D8:E8"/>
     <mergeCell ref="D6:E6"/>
+    <mergeCell ref="D16:E16"/>
     <mergeCell ref="D7:E7"/>
     <mergeCell ref="D10:E10"/>
-    <mergeCell ref="D15:E15"/>
-    <mergeCell ref="D19:E19"/>
     <mergeCell ref="D11:E11"/>
     <mergeCell ref="D13:E13"/>
     <mergeCell ref="D17:E17"/>
-    <mergeCell ref="D23:E23"/>
     <mergeCell ref="D14:E14"/>
     <mergeCell ref="D4:E4"/>
-    <mergeCell ref="D22:E22"/>
     <mergeCell ref="D18:E18"/>
     <mergeCell ref="D9:E9"/>
     <mergeCell ref="D12:E12"/>
-    <mergeCell ref="D21:E21"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>

</xml_diff>